<commit_message>
Fix: replace Power Query injection with pure Excel 365 formulas
Power Query XML injection into xlsx was corrupting the file on open.
Rebuilt using native LET/AVERAGEIFS/UNIQUE formulas only — no Power Query,
no macros, no external connections. File opens cleanly and all three lookup
tiers (exact match, extrapolation, geographic fallback) work via formulas
that reference tblData directly.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019F6cSPJfFZ4zUJ6UoDQ6a5
</commit_message>
<xml_diff>
--- a/CSI_Tool.xlsx
+++ b/CSI_Tool.xlsx
@@ -4,29 +4,16 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="PostcodeCoords" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet name="PQ_Summary" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet name="PQ_PostcodeAgg" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet name="Tool" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tool" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
-<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <connection id="1" keepAlive="0" name="Query - CSI_Summary" description="Connection to the Power Query CSI_Summary" type="5" refreshedVersion="0" background="0" saveData="1" refreshOnLoad="1">
-    <dbPr connection="Provider=Microsoft.Mashup.OleDb.1;Data Source=$Workbook$;Location=CSI_Summary" command="SELECT * FROM [CSI_Summary]"/>
-  </connection>
-  <connection id="2" keepAlive="0" name="Query - CSI_PostcodeAgg" description="Connection to the Power Query CSI_PostcodeAgg" type="5" refreshedVersion="0" background="0" saveData="1" refreshOnLoad="1">
-    <dbPr connection="Provider=Microsoft.Mashup.OleDb.1;Data Source=$Workbook$;Location=CSI_PostcodeAgg" command="SELECT * FROM [CSI_PostcodeAgg]"/>
-  </connection>
-</connections>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -34,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="£#,##0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,7 +45,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <b val="1"/>
@@ -68,17 +55,17 @@
     <font>
       <b val="1"/>
       <color rgb="001B2A4A"/>
-      <sz val="13"/>
+      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00555555"/>
-      <sz val="11"/>
+      <color rgb="00444444"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00C9A84C"/>
-      <sz val="24"/>
+      <sz val="26"/>
     </font>
     <font>
       <i val="1"/>
@@ -89,9 +76,6 @@
       <i val="1"/>
       <color rgb="00B0BEC5"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="5">
@@ -113,31 +97,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9E6"/>
+        <fgColor rgb="00FFFDE7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="001B2A4A"/>
-      </left>
-      <right style="thin">
-        <color rgb="001B2A4A"/>
-      </right>
-      <top style="thin">
-        <color rgb="001B2A4A"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="001B2A4A"/>
-      </bottom>
     </border>
     <border>
       <left style="medium">
@@ -154,7 +124,7 @@
       </bottom>
     </border>
     <border>
-      <bottom style="thin">
+      <bottom style="medium">
         <color rgb="00C9A84C"/>
       </bottom>
     </border>
@@ -162,29 +132,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -272,51 +243,9 @@
 </styleSheet>
 </file>
 
-<file path=xl/customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<Workbook xmlns="http://schemas.microsoft.com/DataModel/Query">
-  <Query Name="CSI_Summary">
-    <Formula>let
-    Source = Excel.CurrentWorkbook(){[Name="tblData"]}[Content],
-    ChangedTypes = Table.TransformColumnTypes(Source, {
-        {"Postcode",  type text},
-        {"Bedrooms",  Int64.Type},
-        {"CSI_Value", type number}
-    }),
-    Cleaned = Table.TransformColumns(ChangedTypes, {
-        {"Postcode", each Text.Upper(Text.Trim(_)), type text}
-    }),
-    Grouped = Table.Group(Cleaned, {"Postcode", "Bedrooms"}, {
-        {"AvgCSI", each List.Average([CSI_Value]), type number},
-        {"Count",  each Table.RowCount(_),         Int64.Type}
-    })
-in
-    Grouped</Formula>
-  </Query>
-  <Query Name="CSI_PostcodeAgg">
-    <Formula>let
-    Source = Excel.CurrentWorkbook(){[Name="tblData"]}[Content],
-    ChangedTypes = Table.TransformColumnTypes(Source, {
-        {"Postcode",  type text},
-        {"Bedrooms",  Int64.Type},
-        {"CSI_Value", type number}
-    }),
-    Cleaned = Table.TransformColumns(ChangedTypes, {
-        {"Postcode", each Text.Upper(Text.Trim(_)), type text}
-    }),
-    Grouped = Table.Group(Cleaned, {"Postcode"}, {
-        {"AvgCSI",        each List.Average([CSI_Value]),                           type number},
-        {"AvgBeds",       each List.Average([Bedrooms]),                            type number},
-        {"CSIPerBedroom", each List.Average([CSI_Value]) / List.Average([Bedrooms]),type number}
-    })
-in
-    Grouped</Formula>
-  </Query>
-</Workbook>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblData" displayName="tblData" ref="A2:C17" headerRowCount="1">
-  <autoFilter ref="A2:C17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblData" displayName="tblData" ref="A2:C20" headerRowCount="1">
+  <autoFilter ref="A2:C20"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Postcode"/>
     <tableColumn id="2" name="Bedrooms"/>
@@ -333,32 +262,6 @@
     <tableColumn id="1" name="Postcode"/>
     <tableColumn id="2" name="Lat"/>
     <tableColumn id="3" name="Lon"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblSummary" displayName="tblSummary" ref="A1:D7" headerRowCount="1">
-  <autoFilter ref="A1:D7"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Postcode"/>
-    <tableColumn id="2" name="Bedrooms"/>
-    <tableColumn id="3" name="AvgCSI"/>
-    <tableColumn id="4" name="Count"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblPostcodeAgg" displayName="tblPostcodeAgg" ref="A1:D7" headerRowCount="1">
-  <autoFilter ref="A1:D7"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Postcode"/>
-    <tableColumn id="2" name="AvgCSI"/>
-    <tableColumn id="3" name="AvgBeds"/>
-    <tableColumn id="4" name="CSIPerBedroom"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1"/>
 </table>
@@ -654,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -665,7 +568,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PASTE YOUR DATA BELOW (row 3 onward).  Columns: Postcode | Bedrooms | CSI_Value.  After pasting new data go to  Data &gt; Refresh All  (or Ctrl+Alt+F5).</t>
+          <t>PASTE YOUR DATA BELOW starting at row 3.  Columns: Postcode | Bedrooms | CSI_Value.  Formulas on the Tool sheet update instantly — no refresh needed.</t>
         </is>
       </c>
     </row>
@@ -728,14 +631,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SW1</t>
+          <t>SE3</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>350000</v>
+        <v>220000</v>
       </c>
     </row>
     <row r="7">
@@ -745,10 +648,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>280000</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="8">
@@ -758,36 +661,36 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>320000</v>
+        <v>280000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>85000</v>
+        <v>320000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>92000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="11">
@@ -797,88 +700,127 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>130000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>145000</v>
+        <v>92000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>195000</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>65000</v>
+        <v>145000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>N1</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>90000</v>
+        <v>195000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LS1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>60000</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LS1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="3" t="n">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LS1</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LS1</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="3" t="n">
         <v>85000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LS1</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>115000</v>
       </c>
     </row>
   </sheetData>
@@ -2528,301 +2470,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Postcode</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Bedrooms</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>AvgCSI</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SE3</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" t="n">
-        <v>117500</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>SW1</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" t="n">
-        <v>335000</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" t="n">
-        <v>88500</v>
-      </c>
-      <c r="D4" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>N1</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C5" t="n">
-        <v>145000</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>LS1</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2</v>
-      </c>
-      <c r="C7" t="n">
-        <v>60000</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Postcode</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>AvgCSI</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>AvgBeds</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>CSIPerBedroom</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SE3</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>117500</v>
-      </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="n">
-        <v>39167</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>SW1</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>307500</v>
-      </c>
-      <c r="C3" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D3" t="n">
-        <v>68333</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>102333</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="D4" t="n">
-        <v>44493</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>N1</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>145000</v>
-      </c>
-      <c r="C5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" t="n">
-        <v>48333</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" t="n">
-        <v>32500</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>LS1</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>60000</v>
-      </c>
-      <c r="C7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" t="n">
-        <v>30000</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <tabColor rgb="00C9A84C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E20"/>
+  <dimension ref="B3:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="3" customWidth="1" min="4" max="4"/>
-    <col hidden="1" width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="E1" s="5">
-        <f>UPPER(TRIM(B9))</f>
-        <v/>
-      </c>
-    </row>
+    <row r="1" ht="20" customHeight="1"/>
     <row r="2" ht="20" customHeight="1"/>
-    <row r="3" ht="32" customHeight="1">
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Contents Sum Insured Lookup Tool</t>
+    <row r="3" ht="34" customHeight="1">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Contents Sum Insured  ·  Lookup Tool</t>
         </is>
       </c>
     </row>
@@ -2830,87 +2496,82 @@
     <row r="5" ht="20" customHeight="1"/>
     <row r="6" ht="20" customHeight="1"/>
     <row r="7" ht="20" customHeight="1"/>
-    <row r="8" ht="26" customHeight="1">
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Postcode Area (e.g. SE3, SW1A)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Postcode Area  (e.g. SE3, SW1A, M1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>SE3</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="7" t="inlineStr">
+    <row r="10" ht="8" customHeight="1"/>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Number of Bedrooms</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="B11" s="8" t="n">
+    <row r="12" ht="34" customHeight="1">
+      <c r="B12" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Suggested Contents Sum Insured</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="50" customHeight="1">
-      <c r="B14" s="11">
-        <f>LET(pc,UPPER(TRIM(B9)),beds,B11,exact,IFERROR(AVERAGEIFS(tblSummary[AvgCSI],tblSummary[Postcode],pc,tblSummary[Bedrooms],beds),0),pc_rate,IFERROR(XLOOKUP(pc,tblPostcodeAgg[Postcode],tblPostcodeAgg[CSIPerBedroom],0),0),tier2,pc_rate*beds,tlat,IFERROR(XLOOKUP(pc,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lat],NA()),NA()),tlon,IFERROR(XLOOKUP(pc,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lon],NA()),NA()),avail,UNIQUE(tblSummary[Postcode]),alat,XLOOKUP(avail,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lat],0),alon,XLOOKUP(avail,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lon],0),dists,(alat-tlat)^2+(alon-tlon)^2,nearest,INDEX(avail,MATCH(MIN(dists),dists,0)),near_exact,IFERROR(AVERAGEIFS(tblSummary[AvgCSI],tblSummary[Postcode],nearest,tblSummary[Bedrooms],beds),0),near_rate,IFERROR(XLOOKUP(nearest,tblPostcodeAgg[Postcode],tblPostcodeAgg[CSIPerBedroom],0),0),near_tier,IF(near_exact&gt;0,near_exact,near_rate*beds),IF(exact&gt;0,exact,IF(tier2&gt;0,tier2,near_tier)))</f>
+    <row r="13" ht="20" customHeight="1"/>
+    <row r="14" ht="14" customHeight="1">
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Average Contents Sum Insured</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="B16" s="10">
+        <f>LET(pc,UPPER(TRIM(B9)),beds,B12,exact,IFERROR(AVERAGEIFS(tblData[CSI_Value],tblData[Postcode],pc,tblData[Bedrooms],beds),0),pc_csi,IFERROR(AVERAGEIF(tblData[Postcode],pc,tblData[CSI_Value]),0),pc_beds,IFERROR(AVERAGEIF(tblData[Postcode],pc,tblData[Bedrooms]),0),tier2,IF(pc_beds&gt;0,pc_csi/pc_beds*beds,0),avail,IFERROR(UNIQUE(tblData[Postcode]),{""}),tlat,IFERROR(XLOOKUP(pc,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lat],NA()),NA()),tlon,IFERROR(XLOOKUP(pc,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lon],NA()),NA()),alat,XLOOKUP(avail,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lat],0),alon,XLOOKUP(avail,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lon],0),dists,(alat-tlat)^2+(alon-tlon)^2,nearest,IFERROR(INDEX(avail,MATCH(MIN(dists),dists,0)),""),n_exact,IFERROR(AVERAGEIFS(tblData[CSI_Value],tblData[Postcode],nearest,tblData[Bedrooms],beds),0),n_csi,IFERROR(AVERAGEIF(tblData[Postcode],nearest,tblData[CSI_Value]),0),n_beds,IFERROR(AVERAGEIF(tblData[Postcode],nearest,tblData[Bedrooms]),0),near_val,IF(n_exact&gt;0,n_exact,IF(n_beds&gt;0,n_csi/n_beds*beds,0)),IF(exact&gt;0,exact,IF(tier2&gt;0,tier2,near_val)))</f>
         <v/>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1"/>
-    <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="12">
-        <f>LET(pc,UPPER(TRIM(B9)),beds,B11,cnt,IFERROR(XLOOKUP(1,(tblSummary[Postcode]=pc)*(tblSummary[Bedrooms]=beds),tblSummary[Count],0),0),IF(cnt&gt;0,"Based on "&amp;TEXT(cnt,"#,##0")&amp;" similar properties","Estimated — no exact match found for this postcode/bedroom combination"))</f>
+    <row r="17" ht="20" customHeight="1"/>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="11">
+        <f>LET(pc,UPPER(TRIM(B9)),beds,B12,cnt,IFERROR(COUNTIFS(tblData[Postcode],pc,tblData[Bedrooms],beds),0),IF(cnt&gt;0,"Based on "&amp;TEXT(cnt,"#,##0")&amp;" similar properties in your data",IF(IFERROR(COUNTIF(tblData[Postcode],pc),0)&gt;0,"No exact bedroom match — figure extrapolated from postcode average","Postcode not in dataset — figure taken from nearest geographic area")))</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1"/>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="13">
-        <f>LET(pc,UPPER(TRIM(B9)),beds,B11,in_summary,COUNTIF(tblSummary[Postcode],pc)&gt;0,exact_match,IFERROR(AVERAGEIFS(tblSummary[AvgCSI],tblSummary[Postcode],pc,tblSummary[Bedrooms],beds),0)&gt;0,tlat,IFERROR(XLOOKUP(pc,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lat],NA()),NA()),tlon,IFERROR(XLOOKUP(pc,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lon],NA()),NA()),avail,UNIQUE(tblSummary[Postcode]),alat,XLOOKUP(avail,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lat],0),alon,XLOOKUP(avail,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lon],0),dists,(alat-tlat)^2+(alon-tlon)^2,nearest,IFERROR(INDEX(avail,MATCH(MIN(dists),dists,0)),""),IF(exact_match,"✓ Exact match",IF(in_summary,"~ Estimated by extrapolating postcode average",IF(nearest&lt;&gt;"","⚠ Postcode not in data — using nearest area: "&amp;nearest,"⚠ No data available"))))</f>
+    <row r="19" ht="20" customHeight="1"/>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="12">
+        <f>LET(pc,UPPER(TRIM(B9)),beds,B12,exact_cnt,IFERROR(COUNTIFS(tblData[Postcode],pc,tblData[Bedrooms],beds),0),pc_cnt,IFERROR(COUNTIF(tblData[Postcode],pc),0),avail,IFERROR(UNIQUE(tblData[Postcode]),{""}),tlat,IFERROR(XLOOKUP(pc,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lat],NA()),NA()),tlon,IFERROR(XLOOKUP(pc,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lon],NA()),NA()),alat,XLOOKUP(avail,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lat],0),alon,XLOOKUP(avail,tblPostcodeCoords[Postcode],tblPostcodeCoords[Lon],0),dists,(alat-tlat)^2+(alon-tlon)^2,nearest,IFERROR(INDEX(avail,MATCH(MIN(dists),dists,0)),""),IF(exact_cnt&gt;0,"✓ Exact match",IF(pc_cnt&gt;0,"~ Extrapolated from postcode area average",IF(nearest&lt;&gt;"","⚠ Using nearest area: "&amp;nearest,"⚠ No data available"))))</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1"/>
-    <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>For internal use only. Data refreshed from the Data sheet.</t>
-        </is>
-      </c>
-    </row>
     <row r="21" ht="20" customHeight="1"/>
-    <row r="22" ht="20" customHeight="1"/>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>For internal use only  ·  Data sourced from the Data sheet</t>
+        </is>
+      </c>
+    </row>
     <row r="23" ht="20" customHeight="1"/>
     <row r="24" ht="20" customHeight="1"/>
     <row r="25" ht="20" customHeight="1"/>
-    <row r="26" ht="20" customHeight="1"/>
-    <row r="27" ht="20" customHeight="1"/>
-    <row r="28" ht="20" customHeight="1"/>
-    <row r="29" ht="20" customHeight="1"/>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="B13:C13"/>
+  <mergeCells count="5">
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B22:C22"/>
     <mergeCell ref="B18:C18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>